<commit_message>
Remove personal_priority feature completely
Database:
- Migration 20261006153000: Drop personal_priority column and priority_enum
- Regenerated TypeScript types (no priority)

Code changes:
- PersonalDataPanel: Remove priority dropdown
- ReadingDashboardPage: Remove priority badges, update comments
- useReadingDashboard: Remove priority from ReadingBook type, remove priority sorting
- useReadingStatus: Remove priority from UpdateReadingStatusParams

Test updates:
- PersonalDataPanel.test.tsx: Remove priority tests (16 tests passing)
- useReadingDashboard.test.tsx: Replace priority tests with title sorting (5 tests passing)
- ReadingDashboardPage.test.tsx: Remove priority badge expectations (9 tests passing)

All 459 tests passing (35 skipped). Reading status + rating is sufficient.

Still TODO: Update specs/docs to remove priority requirements

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/migration/test-data.xlsx
+++ b/migration/test-data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,22 +416,22 @@
         <v>Category</v>
       </c>
       <c r="F1" t="str">
+        <v>Read</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Last Name</v>
+      </c>
+      <c r="H1" t="str">
+        <v>First Name</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Genre</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Lib</v>
+      </c>
+      <c r="K1" t="str">
         <v>Prio</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Read</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Last Name</v>
-      </c>
-      <c r="I1" t="str">
-        <v>First Name</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Genre</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Lib</v>
       </c>
     </row>
     <row r="2">
@@ -451,9 +451,6 @@
         <v>Epic</v>
       </c>
       <c r="F2" t="str">
-        <v>x</v>
-      </c>
-      <c r="G2" t="str">
         <v>X</v>
       </c>
     </row>
@@ -467,33 +464,44 @@
       <c r="D3">
         <v>1869</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
+        <v>Tolstoy</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Leo</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Historical Fiction</v>
+      </c>
+      <c r="J3" t="str">
+        <v>X</v>
+      </c>
+      <c r="K3" t="str">
         <v>5</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Tolstoy</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Leo</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Historical Fiction</v>
-      </c>
-      <c r="K3" t="str">
-        <v>X</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Kafka</v>
+      </c>
+      <c r="B4" t="str">
+        <v>The Trial</v>
+      </c>
+      <c r="K4" t="str">
+        <v>x</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>Unknown</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v>Beowulf</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>